<commit_message>
so do gia thuat
</commit_message>
<xml_diff>
--- a/09_02.xlsx
+++ b/09_02.xlsx
@@ -5,16 +5,17 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DuLieuCua_Sang\HK261\Testing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DuLieuCua_Sang\HK261\Testing\Project\09_02\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{633AFC41-8C34-4F26-8F3B-0B732E20AB42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D419A33-AE3A-42D3-B467-105CDC836924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{24A087C9-FC7B-41A3-BD57-B9096DC3F569}"/>
   </bookViews>
   <sheets>
     <sheet name="0. Cover Page" sheetId="1" r:id="rId1"/>
     <sheet name="1. White Box" sheetId="2" r:id="rId2"/>
+    <sheet name="2. JUnit Test Result" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>ĐỒ ÁN CUỐI KÌ</t>
   </si>
@@ -70,9 +71,6 @@
     <t>khanh.2474801030029@vanlanguni.vn</t>
   </si>
   <si>
-    <t>TÍNH GIÁ VÉ MÁY BAY</t>
-  </si>
-  <si>
     <t>Testcase ID</t>
   </si>
   <si>
@@ -95,6 +93,21 @@
   </si>
   <si>
     <t xml:space="preserve">Bảng quyết định só 1 </t>
+  </si>
+  <si>
+    <t>Đề 2: TÍNH GIÁ VÉ MÁY BAY</t>
+  </si>
+  <si>
+    <t>TC_01: giải thích cột nào của bảng quyết định</t>
+  </si>
+  <si>
+    <t>20% test case fail</t>
+  </si>
+  <si>
+    <t>Chuoj hình kết quả các testcases Failed</t>
+  </si>
+  <si>
+    <t>Xuất toàn bộ kết quả ra file JUnitTestResult.csv</t>
   </si>
 </sst>
 </file>
@@ -184,6 +197,61 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>120650</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>482600</xdr:colOff>
+      <xdr:row>141</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DE935882-067B-13CD-6517-9CD6146D96A9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7156450" y="95250"/>
+          <a:ext cx="8286750" cy="25869900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -568,7 +636,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F7F2656-C2F3-45D0-B2D5-24D480F4A636}">
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:Y10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.54296875" customWidth="1"/>
@@ -577,70 +645,98 @@
     <col min="4" max="4" width="17.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="O1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
+      <c r="B2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E2" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="E5" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
     </row>
+    <row r="10" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7D49E8C-3D16-4DF4-BEED-63520DF02D1C}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>26</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>